<commit_message>
updated BOm to v3.0, created gerber files
</commit_message>
<xml_diff>
--- a/production/BOM/BOM_ZumoComSystem.xlsx
+++ b/production/BOM/BOM_ZumoComSystem.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nschneider\Documents\NT_Projekte\ZumoComSystemHW\production\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78ABEBF1-7825-4B4E-B612-F6FB0BA65D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4961ED0A-7CFC-4143-9EAA-7C25AF703904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="5085" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="218">
   <si>
     <t>ZumoComSystem</t>
   </si>
@@ -42,9 +42,6 @@
     <t>C3216X5R1V226M160AC</t>
   </si>
   <si>
-    <t>C3216X5R1A107M160AC</t>
-  </si>
-  <si>
     <t>TDK Corporation</t>
   </si>
   <si>
@@ -60,9 +57,6 @@
     <t>30V 100mA</t>
   </si>
   <si>
-    <t>1050570001</t>
-  </si>
-  <si>
     <t>Battery_Cell</t>
   </si>
   <si>
@@ -78,12 +72,6 @@
     <t>CC0603JRX7R9BB104</t>
   </si>
   <si>
-    <t>1u</t>
-  </si>
-  <si>
-    <t>C1608X5R1H105M080AB</t>
-  </si>
-  <si>
     <t>330n</t>
   </si>
   <si>
@@ -126,21 +114,12 @@
     <t>150060SS55040</t>
   </si>
   <si>
-    <t xml:space="preserve">    D8</t>
-  </si>
-  <si>
     <t>LED, green</t>
   </si>
   <si>
     <t>150060VS55040</t>
   </si>
   <si>
-    <t xml:space="preserve">    D9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    D10</t>
-  </si>
-  <si>
     <t>Broadcom Limited</t>
   </si>
   <si>
@@ -156,36 +135,18 @@
     <t xml:space="preserve">    J1</t>
   </si>
   <si>
-    <t>USB_A_Molex_105057</t>
-  </si>
-  <si>
     <t>Molex</t>
   </si>
   <si>
-    <t>USB_B_Micro</t>
-  </si>
-  <si>
-    <t>1051330001</t>
-  </si>
-  <si>
     <t>Samtec</t>
   </si>
   <si>
-    <t>TSM-113-01-T-DV</t>
-  </si>
-  <si>
     <t xml:space="preserve">    J5</t>
   </si>
   <si>
-    <t>Conn_02x07_Odd_Even</t>
-  </si>
-  <si>
     <t xml:space="preserve">    J7</t>
   </si>
   <si>
-    <t>SSM-107-T-DV-P</t>
-  </si>
-  <si>
     <t xml:space="preserve">    L1</t>
   </si>
   <si>
@@ -195,21 +156,9 @@
     <t>Rohm Semiconductor</t>
   </si>
   <si>
-    <t>&gt;  Q2, Q3</t>
-  </si>
-  <si>
     <t>RQ5E065AJTCL</t>
   </si>
   <si>
-    <t>NPN-SS8050</t>
-  </si>
-  <si>
-    <t>Comchip Technology</t>
-  </si>
-  <si>
-    <t>SS8050-G</t>
-  </si>
-  <si>
     <t>SI2302CDS-T1-BE3</t>
   </si>
   <si>
@@ -243,12 +192,6 @@
     <t>RC0603FR-072KL</t>
   </si>
   <si>
-    <t>12k</t>
-  </si>
-  <si>
-    <t>CRGCQ0603F12K</t>
-  </si>
-  <si>
     <t>4.93k / 0.1%</t>
   </si>
   <si>
@@ -300,15 +243,6 @@
     <t>Part-No.</t>
   </si>
   <si>
-    <t xml:space="preserve">    J7*</t>
-  </si>
-  <si>
-    <t>Erhöhung von J7</t>
-  </si>
-  <si>
-    <t>ESQ-107-13-T-D</t>
-  </si>
-  <si>
     <t>RC1206FR-070RL</t>
   </si>
   <si>
@@ -348,18 +282,9 @@
     <t>100u</t>
   </si>
   <si>
-    <t>Pin-Header 2x13</t>
-  </si>
-  <si>
     <t>15u</t>
   </si>
   <si>
-    <t xml:space="preserve"> Vishay / Dale </t>
-  </si>
-  <si>
-    <t>IHLP4040DZER150M5A</t>
-  </si>
-  <si>
     <t xml:space="preserve">Taiwan Semiconductor </t>
   </si>
   <si>
@@ -369,24 +294,9 @@
     <t>10k / 0.1%</t>
   </si>
   <si>
-    <t xml:space="preserve">   J4*, J6*</t>
-  </si>
-  <si>
-    <t>Pin-Socket 2x13 for Zumo Robot</t>
-  </si>
-  <si>
-    <t>SSQ-113-01-T-D</t>
-  </si>
-  <si>
     <t>LED, yellow</t>
   </si>
   <si>
-    <t xml:space="preserve">    Q7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    R21</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Kyocera AVX </t>
   </si>
   <si>
@@ -408,12 +318,6 @@
     <t xml:space="preserve">Keystone Electronics </t>
   </si>
   <si>
-    <t>&gt;  C1, C3, C4</t>
-  </si>
-  <si>
-    <t>&gt;  C2, C5, C7</t>
-  </si>
-  <si>
     <t>Samsung Electro-Mechanics</t>
   </si>
   <si>
@@ -426,36 +330,15 @@
     <t xml:space="preserve">    C8</t>
   </si>
   <si>
-    <t xml:space="preserve">    C9</t>
-  </si>
-  <si>
     <t xml:space="preserve">    C10</t>
   </si>
   <si>
-    <t>&gt;  C11, C14</t>
-  </si>
-  <si>
-    <t>Kemet</t>
-  </si>
-  <si>
-    <t>T491A106K020AT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    C12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    C13</t>
-  </si>
-  <si>
     <t>LED_ARGB</t>
   </si>
   <si>
     <t xml:space="preserve">    D4</t>
   </si>
   <si>
-    <t>&gt;  D5-D7, D11-D13</t>
-  </si>
-  <si>
     <t>40V/2A</t>
   </si>
   <si>
@@ -477,21 +360,9 @@
     <t xml:space="preserve">    D15</t>
   </si>
   <si>
-    <t xml:space="preserve">    D16</t>
-  </si>
-  <si>
-    <t>1N5819HW1-7-F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    IC1</t>
-  </si>
-  <si>
     <t>ABLIC</t>
   </si>
   <si>
-    <t xml:space="preserve">    IC2</t>
-  </si>
-  <si>
     <t>MCP73844-840I_MS</t>
   </si>
   <si>
@@ -501,15 +372,9 @@
     <t>MCP73844T-840I/MS</t>
   </si>
   <si>
-    <t>&gt;  J2, J3</t>
-  </si>
-  <si>
     <t xml:space="preserve">    J4</t>
   </si>
   <si>
-    <t>TSW-107-07-T-D</t>
-  </si>
-  <si>
     <t xml:space="preserve">    J6</t>
   </si>
   <si>
@@ -519,9 +384,6 @@
     <t>CUI Devices</t>
   </si>
   <si>
-    <t xml:space="preserve">    Q4</t>
-  </si>
-  <si>
     <t>Q_PMOS_GSD</t>
   </si>
   <si>
@@ -531,12 +393,6 @@
     <t>TSM500P02CX RFG</t>
   </si>
   <si>
-    <t>&gt;  Q5, Q6</t>
-  </si>
-  <si>
-    <t>&gt;  R1, R5, R6, R10, R11, R14, R15, R31</t>
-  </si>
-  <si>
     <t xml:space="preserve">    R2</t>
   </si>
   <si>
@@ -549,12 +405,6 @@
     <t xml:space="preserve">CR0603-FX-6200ELF </t>
   </si>
   <si>
-    <t>&gt;  R12, R13, R18</t>
-  </si>
-  <si>
-    <t>&gt;  R16, R17</t>
-  </si>
-  <si>
     <t>100k</t>
   </si>
   <si>
@@ -564,9 +414,6 @@
     <t>RMCF0603FT100K</t>
   </si>
   <si>
-    <t xml:space="preserve">    R20</t>
-  </si>
-  <si>
     <t>220m</t>
   </si>
   <si>
@@ -576,9 +423,6 @@
     <t xml:space="preserve">ERJ-6RQFR22V </t>
   </si>
   <si>
-    <t xml:space="preserve">    R22</t>
-  </si>
-  <si>
     <t xml:space="preserve">    R23</t>
   </si>
   <si>
@@ -588,42 +432,12 @@
     <t xml:space="preserve">    R25</t>
   </si>
   <si>
-    <t>&gt;  R26, R27</t>
-  </si>
-  <si>
     <t xml:space="preserve">    R28</t>
   </si>
   <si>
-    <t>22.1k / 0.1%</t>
-  </si>
-  <si>
-    <t>KOA Speer</t>
-  </si>
-  <si>
-    <t>RN73H1JTTD2212B25</t>
-  </si>
-  <si>
     <t xml:space="preserve">    R29</t>
   </si>
   <si>
-    <t>47.5k / 0.5%</t>
-  </si>
-  <si>
-    <t>RN73H1JTTD4752D50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    R30</t>
-  </si>
-  <si>
-    <t>1k</t>
-  </si>
-  <si>
-    <t>Vishay / Draloric</t>
-  </si>
-  <si>
-    <t>RCA04021K00JNED</t>
-  </si>
-  <si>
     <t>User_Button</t>
   </si>
   <si>
@@ -645,18 +459,6 @@
     <t>espressif</t>
   </si>
   <si>
-    <t>CP2102N-Axx-xQFN28</t>
-  </si>
-  <si>
-    <t>Silicon Laboratories Inc.</t>
-  </si>
-  <si>
-    <t>LM1117MP-3.3</t>
-  </si>
-  <si>
-    <t>v2.0</t>
-  </si>
-  <si>
     <t>&gt;  SW2-SW5, SW7</t>
   </si>
   <si>
@@ -666,14 +468,250 @@
     <t>PMOS_GSD-TSM260P02CX RFG</t>
   </si>
   <si>
-    <t xml:space="preserve"> Texas Instruments </t>
+    <t>v3.0</t>
+  </si>
+  <si>
+    <t>&gt;  C1, C12, C15</t>
+  </si>
+  <si>
+    <t>&gt;  C2, C7, C9, C11, C13, C14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    C3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    C4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    C5</t>
+  </si>
+  <si>
+    <t>2.2u</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Murata Electronics </t>
+  </si>
+  <si>
+    <t>GRM188R61H225KE11D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KYOCERA AVX </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TPSD107K016R0060 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRM21BR61E226ME44K </t>
+  </si>
+  <si>
+    <t xml:space="preserve">    C16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    D5</t>
+  </si>
+  <si>
+    <t>&gt;  D6, D9, D10</t>
+  </si>
+  <si>
+    <t>20V 1A</t>
+  </si>
+  <si>
+    <t>SD0805S020S1R0</t>
+  </si>
+  <si>
+    <t>&gt;  D7, D8</t>
+  </si>
+  <si>
+    <t>SD03C-7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    D11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    D12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    D13</t>
+  </si>
+  <si>
+    <t>USB_C_Receptacle_USB2.0_16P</t>
+  </si>
+  <si>
+    <t>2171820001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    J2</t>
+  </si>
+  <si>
+    <t>Conn_02x11_Odd_Even</t>
+  </si>
+  <si>
+    <t>TSM-111-01-T-DV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    J3</t>
+  </si>
+  <si>
+    <t>Conn_02x05_Odd_Even</t>
+  </si>
+  <si>
+    <t>SSM-105-T-DV</t>
+  </si>
+  <si>
+    <t>Conn_02x14_Odd_Even</t>
+  </si>
+  <si>
+    <t>TSM-114-01-T-DV</t>
+  </si>
+  <si>
+    <t>Conn_01x07</t>
+  </si>
+  <si>
+    <t>TSM-107-01-T-SV</t>
+  </si>
+  <si>
+    <t>SSM-107-T-SV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRP7050WA-220M </t>
+  </si>
+  <si>
+    <t xml:space="preserve">    L2</t>
+  </si>
+  <si>
+    <t>TDK</t>
+  </si>
+  <si>
+    <t>BCL322515RT-150M-D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Q2</t>
+  </si>
+  <si>
+    <t>&gt;  Q3, Q4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Q5</t>
+  </si>
+  <si>
+    <t>&gt;  R1, R5, R6, R10, R11, R16, R17</t>
+  </si>
+  <si>
+    <t>&gt;  R12, R13</t>
+  </si>
+  <si>
+    <t>4.7k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RT0603FRE134K7L </t>
+  </si>
+  <si>
+    <t>&gt;  R14, R15, R22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    R18</t>
+  </si>
+  <si>
+    <t>51k</t>
+  </si>
+  <si>
+    <t>RT0603BRD0751KL</t>
+  </si>
+  <si>
+    <t>22.1k</t>
+  </si>
+  <si>
+    <t>RT0603BRD0722K1L</t>
+  </si>
+  <si>
+    <t>&gt;  R20, R21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    R26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    R27</t>
+  </si>
+  <si>
+    <t>TPS560430X3FDBVR</t>
+  </si>
+  <si>
+    <t>Texas Instruments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    U5</t>
+  </si>
+  <si>
+    <t>SSQ-111-21-F-D</t>
+  </si>
+  <si>
+    <t>SSQ-114-21-F-D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    J2*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    J4*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    J3*</t>
+  </si>
+  <si>
+    <t>ESQ-105-38-T-D</t>
+  </si>
+  <si>
+    <t>ESQ-107-38-T-S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    J6*</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Pin-Socket 2x11 for </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Zumo Robot</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Pin-Socket 2x14 for </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Zumo Robot</t>
+    </r>
+  </si>
+  <si>
+    <t>Increase in J3</t>
+  </si>
+  <si>
+    <t>Increase in J6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kyocera AVX </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -706,13 +744,33 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -728,7 +786,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
@@ -744,6 +802,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -783,8 +847,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A4:E69" totalsRowShown="0" dataDxfId="5">
-  <autoFilter ref="A4:E69" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A4:E73" totalsRowShown="0" dataDxfId="5">
+  <autoFilter ref="A4:E73" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Reference" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Value" dataDxfId="3"/>
@@ -1079,10 +1143,10 @@
         <v>0</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>125</v>
+        <v>95</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>209</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.35">
@@ -1090,30 +1154,30 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="B4" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="C4" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="D4" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>95</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>86</v>
+        <v>67</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>126</v>
+        <v>96</v>
       </c>
       <c r="D5" s="3">
         <v>1043</v>
@@ -1124,16 +1188,16 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>14</v>
+        <v>78</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>15</v>
+        <v>97</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>16</v>
+        <v>98</v>
       </c>
       <c r="E6" s="5">
         <v>3</v>
@@ -1142,34 +1206,34 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>100</v>
+        <v>12</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>129</v>
+        <v>13</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>130</v>
+        <v>14</v>
       </c>
       <c r="E7" s="5">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H7" s="2"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>19</v>
+        <v>81</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="E8" s="5">
         <v>1</v>
@@ -1178,16 +1242,16 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>17</v>
+        <v>82</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E9" s="5">
         <v>1</v>
@@ -1196,16 +1260,16 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>133</v>
+        <v>152</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>103</v>
+        <v>153</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>101</v>
+        <v>154</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>99</v>
+        <v>155</v>
       </c>
       <c r="E10" s="5">
         <v>1</v>
@@ -1214,16 +1278,16 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>134</v>
+        <v>99</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>104</v>
+        <v>83</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E11" s="5">
         <v>1</v>
@@ -1232,34 +1296,34 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>135</v>
+        <v>100</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="E12" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H12" s="2"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>138</v>
+        <v>101</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>105</v>
+        <v>81</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>7</v>
+        <v>154</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>13</v>
+        <v>158</v>
       </c>
       <c r="E13" s="5">
         <v>1</v>
@@ -1268,16 +1332,16 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>139</v>
+        <v>159</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>106</v>
+        <v>15</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="E14" s="5">
         <v>1</v>
@@ -1286,16 +1350,16 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>140</v>
+        <v>102</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="E15" s="5">
         <v>1</v>
@@ -1304,16 +1368,16 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>117</v>
+        <v>89</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
       <c r="E16" s="5">
         <v>1</v>
@@ -1322,16 +1386,16 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E17" s="5">
         <v>1</v>
@@ -1340,16 +1404,16 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>141</v>
+        <v>103</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E18" s="5">
         <v>1</v>
@@ -1358,70 +1422,70 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>142</v>
+        <v>160</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E19" s="5">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H19" s="2"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>33</v>
+        <v>161</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>143</v>
+        <v>162</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>144</v>
+        <v>90</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="E20" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H20" s="2"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>36</v>
+        <v>164</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>146</v>
+        <v>165</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>147</v>
+        <v>165</v>
       </c>
       <c r="E21" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H21" s="2"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>37</v>
+        <v>166</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>27</v>
+        <v>217</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="E22" s="5">
         <v>1</v>
@@ -1430,16 +1494,16 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>148</v>
+        <v>167</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>120</v>
+        <v>19</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E23" s="5">
         <v>1</v>
@@ -1448,16 +1512,16 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>149</v>
+        <v>168</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>10</v>
+        <v>104</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>23</v>
+        <v>105</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>24</v>
+        <v>106</v>
       </c>
       <c r="E24" s="5">
         <v>1</v>
@@ -1466,16 +1530,16 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>150</v>
+        <v>109</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>151</v>
+        <v>107</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>151</v>
+        <v>108</v>
       </c>
       <c r="E25" s="5">
         <v>1</v>
@@ -1484,16 +1548,16 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>40</v>
+        <v>110</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="E26" s="5">
         <v>1</v>
@@ -1502,16 +1566,16 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>152</v>
+        <v>33</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>85</v>
+        <v>34</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>153</v>
+        <v>1</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>85</v>
+        <v>3</v>
       </c>
       <c r="E27" s="5">
         <v>1</v>
@@ -1520,16 +1584,16 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>154</v>
+        <v>35</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>156</v>
+        <v>36</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="E28" s="5">
         <v>1</v>
@@ -1538,16 +1602,16 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>42</v>
+        <v>171</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>43</v>
+        <v>172</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>11</v>
+        <v>173</v>
       </c>
       <c r="E29" s="5">
         <v>1</v>
@@ -1556,34 +1620,34 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>107</v>
+        <v>175</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>48</v>
+        <v>176</v>
       </c>
       <c r="E30" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H30" s="2"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>159</v>
+        <v>115</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>50</v>
+        <v>177</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="E31" s="5">
         <v>1</v>
@@ -1592,16 +1656,16 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>50</v>
+        <v>179</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>52</v>
+        <v>180</v>
       </c>
       <c r="E32" s="5">
         <v>1</v>
@@ -1610,16 +1674,16 @@
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>161</v>
+        <v>116</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>163</v>
+        <v>37</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>162</v>
+        <v>181</v>
       </c>
       <c r="E33" s="5">
         <v>1</v>
@@ -1628,16 +1692,16 @@
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>45</v>
+        <v>117</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>44</v>
+        <v>118</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>46</v>
+        <v>117</v>
       </c>
       <c r="E34" s="5">
         <v>1</v>
@@ -1646,16 +1710,16 @@
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>108</v>
+        <v>81</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>110</v>
+        <v>182</v>
       </c>
       <c r="E35" s="5">
         <v>1</v>
@@ -1664,16 +1728,16 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>54</v>
+        <v>183</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>62</v>
+        <v>184</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>61</v>
+        <v>185</v>
       </c>
       <c r="E36" s="5">
         <v>1</v>
@@ -1681,34 +1745,34 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="E37" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H37" s="2"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>164</v>
+        <v>186</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>165</v>
+        <v>146</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>166</v>
+        <v>86</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>167</v>
+        <v>87</v>
       </c>
       <c r="E38" s="5">
         <v>1</v>
@@ -1717,16 +1781,16 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>168</v>
+        <v>187</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="E39" s="5">
         <v>2</v>
@@ -1734,16 +1798,16 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>118</v>
+        <v>188</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>212</v>
+        <v>119</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="E40" s="5">
         <v>1</v>
@@ -1751,24 +1815,24 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>169</v>
+        <v>189</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="E41" s="5">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>170</v>
+        <v>122</v>
       </c>
       <c r="B42" s="3">
         <v>300</v>
@@ -1777,7 +1841,7 @@
         <v>1</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="E42" s="5">
         <v>1</v>
@@ -1785,16 +1849,16 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>171</v>
+        <v>123</v>
       </c>
       <c r="B43" s="3">
         <v>100</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
       <c r="E43" s="5">
         <v>2</v>
@@ -1802,16 +1866,16 @@
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>172</v>
+        <v>124</v>
       </c>
       <c r="B44" s="3">
         <v>620</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>124</v>
+        <v>94</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>173</v>
+        <v>125</v>
       </c>
       <c r="E44" s="5">
         <v>3</v>
@@ -1819,50 +1883,50 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="B45" s="3">
-        <v>0</v>
+        <v>190</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>191</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>66</v>
+        <v>192</v>
       </c>
       <c r="E45" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>175</v>
+        <v>193</v>
       </c>
       <c r="B46" s="3">
-        <v>470</v>
+        <v>0</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="E46" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>102</v>
+        <v>194</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>177</v>
+        <v>13</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>178</v>
+        <v>196</v>
       </c>
       <c r="E47" s="5">
         <v>1</v>
@@ -1870,16 +1934,16 @@
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>179</v>
+        <v>80</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>180</v>
+        <v>197</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>181</v>
+        <v>13</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="E48" s="5">
         <v>1</v>
@@ -1887,33 +1951,33 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>119</v>
+        <v>199</v>
       </c>
       <c r="B49" s="3">
-        <v>0</v>
+        <v>470</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>94</v>
+        <v>52</v>
       </c>
       <c r="E49" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>183</v>
+        <v>132</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>70</v>
+        <v>126</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>15</v>
+        <v>127</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>71</v>
+        <v>128</v>
       </c>
       <c r="E50" s="5">
         <v>1</v>
@@ -1921,16 +1985,16 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>184</v>
+        <v>133</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>64</v>
+        <v>130</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>65</v>
+        <v>131</v>
       </c>
       <c r="E51" s="5">
         <v>1</v>
@@ -1938,16 +2002,16 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>74</v>
+        <v>134</v>
+      </c>
+      <c r="B52" s="3">
+        <v>0</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E52" s="5">
         <v>1</v>
@@ -1955,16 +2019,16 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>186</v>
+        <v>200</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="E53" s="5">
         <v>1</v>
@@ -1972,33 +2036,33 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>187</v>
+        <v>201</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>73</v>
+        <v>48</v>
       </c>
       <c r="E54" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>188</v>
+        <v>135</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>189</v>
+        <v>55</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>190</v>
+        <v>13</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>191</v>
+        <v>56</v>
       </c>
       <c r="E55" s="5">
         <v>1</v>
@@ -2006,16 +2070,16 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>192</v>
+        <v>136</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>193</v>
+        <v>50</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>190</v>
+        <v>47</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>194</v>
+        <v>51</v>
       </c>
       <c r="E56" s="5">
         <v>1</v>
@@ -2023,16 +2087,16 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>195</v>
+        <v>58</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>196</v>
+        <v>137</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>197</v>
+        <v>2</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>198</v>
+        <v>59</v>
       </c>
       <c r="E57" s="5">
         <v>1</v>
@@ -2040,50 +2104,50 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>77</v>
+        <v>144</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>199</v>
+        <v>138</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>2</v>
+        <v>139</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>78</v>
+        <v>140</v>
       </c>
       <c r="E58" s="5">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>210</v>
+        <v>141</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>200</v>
+        <v>145</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>201</v>
+        <v>2</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>202</v>
+        <v>145</v>
       </c>
       <c r="E59" s="5">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>203</v>
+        <v>60</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>211</v>
+        <v>142</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>2</v>
+        <v>143</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>211</v>
+        <v>142</v>
       </c>
       <c r="E60" s="5">
         <v>1</v>
@@ -2091,16 +2155,16 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>204</v>
+        <v>61</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>205</v>
+        <v>62</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>204</v>
+        <v>61</v>
       </c>
       <c r="E61" s="5">
         <v>1</v>
@@ -2108,16 +2172,16 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="E62" s="5">
         <v>1</v>
@@ -2125,16 +2189,16 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>81</v>
+        <v>111</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="E63" s="5">
         <v>1</v>
@@ -2142,16 +2206,16 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>84</v>
+        <v>204</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>208</v>
+        <v>112</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>213</v>
+        <v>113</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>208</v>
+        <v>114</v>
       </c>
       <c r="E64" s="5">
         <v>1</v>
@@ -2165,13 +2229,13 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>96</v>
+        <v>74</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>97</v>
+        <v>75</v>
       </c>
       <c r="D66" s="3">
         <v>100833</v>
@@ -2182,16 +2246,16 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>92</v>
+        <v>207</v>
+      </c>
+      <c r="B67" s="9" t="s">
+        <v>213</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D67" s="3" t="s">
-        <v>93</v>
+        <v>37</v>
+      </c>
+      <c r="D67" t="s">
+        <v>205</v>
       </c>
       <c r="E67" s="5">
         <v>1</v>
@@ -2199,36 +2263,75 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>115</v>
+        <v>208</v>
+      </c>
+      <c r="B68" s="9" t="s">
+        <v>214</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D68" s="3" t="s">
-        <v>116</v>
+        <v>37</v>
+      </c>
+      <c r="D68" t="s">
+        <v>206</v>
       </c>
       <c r="E68" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="3"/>
-      <c r="B69" s="3"/>
-      <c r="C69" s="3"/>
-      <c r="D69" s="3"/>
+      <c r="A69" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D69" t="s">
+        <v>210</v>
+      </c>
+      <c r="E69" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D70" t="s">
+        <v>211</v>
+      </c>
+      <c r="E70" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="3"/>
+      <c r="B71" s="3"/>
+      <c r="C71" s="3"/>
+      <c r="D71" s="8"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="3"/>
+      <c r="B72" s="3"/>
+      <c r="C72" s="3"/>
       <c r="D72" s="3"/>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
+      <c r="D73" s="3"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
move gerber files (delete sub folder)
final files (pre order)
</commit_message>
<xml_diff>
--- a/production/BOM/BOM_ZumoComSystem.xlsx
+++ b/production/BOM/BOM_ZumoComSystem.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nschneider\Documents\NT_Projekte\ZumoComSystemHW\production\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4961ED0A-7CFC-4143-9EAA-7C25AF703904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{953BE605-F2BD-4F04-8D15-E36687CF04F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5085" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="217">
   <si>
     <t>ZumoComSystem</t>
   </si>
@@ -297,9 +297,6 @@
     <t>LED, yellow</t>
   </si>
   <si>
-    <t xml:space="preserve"> Kyocera AVX </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Würth Elektronik</t>
   </si>
   <si>
@@ -493,9 +490,6 @@
   </si>
   <si>
     <t>GRM188R61H225KE11D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KYOCERA AVX </t>
   </si>
   <si>
     <t xml:space="preserve">TPSD107K016R0060 </t>
@@ -704,7 +698,10 @@
     <t>Increase in J6</t>
   </si>
   <si>
-    <t xml:space="preserve">Kyocera AVX </t>
+    <t>Kyocera AVX</t>
+  </si>
+  <si>
+    <t>RE0603BRE0710KL</t>
   </si>
 </sst>
 </file>
@@ -1143,10 +1140,10 @@
         <v>0</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.35">
@@ -1177,7 +1174,7 @@
         <v>10</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D5" s="3">
         <v>1043</v>
@@ -1188,16 +1185,16 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>97</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>98</v>
       </c>
       <c r="E6" s="5">
         <v>3</v>
@@ -1206,7 +1203,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>12</v>
@@ -1224,7 +1221,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>81</v>
@@ -1242,7 +1239,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>82</v>
@@ -1260,16 +1257,16 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="4" t="s">
         <v>154</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>155</v>
       </c>
       <c r="E10" s="5">
         <v>1</v>
@@ -1278,7 +1275,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>83</v>
@@ -1296,16 +1293,16 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>84</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>156</v>
+        <v>215</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E12" s="5">
         <v>1</v>
@@ -1314,16 +1311,16 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>81</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E13" s="5">
         <v>1</v>
@@ -1332,7 +1329,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>15</v>
@@ -1353,7 +1350,7 @@
         <v>17</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>31</v>
@@ -1374,10 +1371,10 @@
         <v>89</v>
       </c>
       <c r="C16" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>91</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>92</v>
       </c>
       <c r="E16" s="5">
         <v>1</v>
@@ -1392,7 +1389,7 @@
         <v>29</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>30</v>
@@ -1404,13 +1401,13 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>27</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>28</v>
@@ -1422,7 +1419,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>25</v>
@@ -1440,16 +1437,16 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D20" s="4" t="s">
         <v>161</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>163</v>
       </c>
       <c r="E20" s="5">
         <v>3</v>
@@ -1458,16 +1455,16 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>26</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E21" s="5">
         <v>2</v>
@@ -1476,13 +1473,13 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>7</v>
@@ -1494,7 +1491,7 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>9</v>
@@ -1512,16 +1509,16 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B24" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="D24" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>106</v>
       </c>
       <c r="E24" s="5">
         <v>1</v>
@@ -1530,16 +1527,16 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E25" s="5">
         <v>1</v>
@@ -1548,7 +1545,7 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>22</v>
@@ -1587,13 +1584,13 @@
         <v>35</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>36</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E28" s="5">
         <v>1</v>
@@ -1602,16 +1599,16 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E29" s="5">
         <v>1</v>
@@ -1620,16 +1617,16 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E30" s="5">
         <v>1</v>
@@ -1638,16 +1635,16 @@
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E31" s="5">
         <v>1</v>
@@ -1659,13 +1656,13 @@
         <v>38</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="E32" s="5">
         <v>1</v>
@@ -1674,16 +1671,16 @@
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E33" s="5">
         <v>1</v>
@@ -1695,13 +1692,13 @@
         <v>39</v>
       </c>
       <c r="B34" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C34" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="C34" s="3" t="s">
-        <v>118</v>
-      </c>
       <c r="D34" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E34" s="5">
         <v>1</v>
@@ -1716,10 +1713,10 @@
         <v>81</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E35" s="5">
         <v>1</v>
@@ -1728,16 +1725,16 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>85</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="E36" s="5">
         <v>1</v>
@@ -1763,10 +1760,10 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>86</v>
@@ -1781,7 +1778,7 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>43</v>
@@ -1798,16 +1795,16 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B40" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C40" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="D40" s="3" t="s">
         <v>120</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>121</v>
       </c>
       <c r="E40" s="5">
         <v>1</v>
@@ -1815,7 +1812,7 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>46</v>
@@ -1832,7 +1829,7 @@
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B42" s="3">
         <v>300</v>
@@ -1849,7 +1846,7 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B43" s="3">
         <v>100</v>
@@ -1858,7 +1855,7 @@
         <v>13</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E43" s="5">
         <v>2</v>
@@ -1866,16 +1863,16 @@
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B44" s="3">
         <v>620</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E44" s="5">
         <v>3</v>
@@ -1883,16 +1880,16 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E45" s="5">
         <v>2</v>
@@ -1900,7 +1897,7 @@
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B46" s="3">
         <v>0</v>
@@ -1917,16 +1914,16 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="E47" s="5">
         <v>1</v>
@@ -1937,13 +1934,13 @@
         <v>80</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E48" s="5">
         <v>1</v>
@@ -1951,7 +1948,7 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B49" s="3">
         <v>470</v>
@@ -1968,16 +1965,16 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B50" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C50" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="C50" s="3" t="s">
+      <c r="D50" s="3" t="s">
         <v>127</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>128</v>
       </c>
       <c r="E50" s="5">
         <v>1</v>
@@ -1985,16 +1982,16 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B51" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C51" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C51" s="3" t="s">
+      <c r="D51" s="3" t="s">
         <v>130</v>
-      </c>
-      <c r="D51" s="3" t="s">
-        <v>131</v>
       </c>
       <c r="E51" s="5">
         <v>1</v>
@@ -2002,7 +1999,7 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B52" s="3">
         <v>0</v>
@@ -2019,7 +2016,7 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>53</v>
@@ -2036,16 +2033,16 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>48</v>
+        <v>216</v>
       </c>
       <c r="E54" s="5">
         <v>1</v>
@@ -2053,7 +2050,7 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>55</v>
@@ -2070,7 +2067,7 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B56" s="3" t="s">
         <v>50</v>
@@ -2090,7 +2087,7 @@
         <v>58</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C57" s="3" t="s">
         <v>2</v>
@@ -2104,16 +2101,16 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B58" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C58" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="C58" s="3" t="s">
+      <c r="D58" s="3" t="s">
         <v>139</v>
-      </c>
-      <c r="D58" s="3" t="s">
-        <v>140</v>
       </c>
       <c r="E58" s="5">
         <v>5</v>
@@ -2121,16 +2118,16 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E59" s="5">
         <v>1</v>
@@ -2141,13 +2138,13 @@
         <v>60</v>
       </c>
       <c r="B60" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C60" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="C60" s="3" t="s">
-        <v>143</v>
-      </c>
       <c r="D60" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E60" s="5">
         <v>1</v>
@@ -2175,13 +2172,13 @@
         <v>64</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="E62" s="5">
         <v>1</v>
@@ -2195,7 +2192,7 @@
         <v>66</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>66</v>
@@ -2206,16 +2203,16 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B64" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C64" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="C64" s="3" t="s">
+      <c r="D64" s="3" t="s">
         <v>113</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>114</v>
       </c>
       <c r="E64" s="5">
         <v>1</v>
@@ -2246,16 +2243,16 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C67" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D67" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="E67" s="5">
         <v>1</v>
@@ -2263,16 +2260,16 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B68" s="9" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C68" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D68" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="E68" s="5">
         <v>1</v>
@@ -2280,16 +2277,16 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C69" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D69" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E69" s="5">
         <v>1</v>
@@ -2297,16 +2294,16 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C70" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D70" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="E70" s="5">
         <v>1</v>

</xml_diff>

<commit_message>
BOM updated to v3.1
</commit_message>
<xml_diff>
--- a/production/BOM/BOM_ZumoComSystem.xlsx
+++ b/production/BOM/BOM_ZumoComSystem.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nschneider\Documents\NT_Projekte\ZumoComSystemHW\production\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{961C1957-7EB4-4193-98D8-F9708F7DD717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{039860A7-7E00-43B3-AD2F-0843C50EB621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="212">
   <si>
     <t>ZumoComSystem</t>
   </si>
@@ -75,21 +75,6 @@
     <t>C1608X5R1H334M080AB</t>
   </si>
   <si>
-    <t xml:space="preserve">    D1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    D2</t>
-  </si>
-  <si>
-    <t>SMC Diode Solutions</t>
-  </si>
-  <si>
-    <t>SD103BWSA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    D3</t>
-  </si>
-  <si>
     <t>8.55VWM 14.5VC</t>
   </si>
   <si>
@@ -123,33 +108,15 @@
     <t>HSMF-C118</t>
   </si>
   <si>
-    <t xml:space="preserve">    F1</t>
-  </si>
-  <si>
     <t>12V / 4.5A</t>
   </si>
   <si>
-    <t xml:space="preserve">    J1</t>
-  </si>
-  <si>
     <t>Molex</t>
   </si>
   <si>
     <t>Samtec</t>
   </si>
   <si>
-    <t xml:space="preserve">    J5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    J7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    L1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Q1</t>
-  </si>
-  <si>
     <t>Rohm Semiconductor</t>
   </si>
   <si>
@@ -198,36 +165,18 @@
     <t>CR0603-JW-301ELF</t>
   </si>
   <si>
-    <t xml:space="preserve">    SW1</t>
-  </si>
-  <si>
     <t>TL3342F260QG</t>
   </si>
   <si>
-    <t xml:space="preserve">    U1</t>
-  </si>
-  <si>
     <t>LT1374CS8-5PBF</t>
   </si>
   <si>
     <t>Analog Device</t>
   </si>
   <si>
-    <t xml:space="preserve">    U2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    U3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    U4</t>
-  </si>
-  <si>
     <t>S-8252AAL-M6T1U</t>
   </si>
   <si>
-    <t>&gt;  BT1, BT2</t>
-  </si>
-  <si>
     <t>Reference</t>
   </si>
   <si>
@@ -264,9 +213,6 @@
     <t xml:space="preserve"> Murata Electronics </t>
   </si>
   <si>
-    <t xml:space="preserve">    R19</t>
-  </si>
-  <si>
     <t>22u</t>
   </si>
   <si>
@@ -318,21 +264,9 @@
     <t>CL31A106KBHNNNE</t>
   </si>
   <si>
-    <t xml:space="preserve">    C6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    C8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    C10</t>
-  </si>
-  <si>
     <t>LED_ARGB</t>
   </si>
   <si>
-    <t xml:space="preserve">    D4</t>
-  </si>
-  <si>
     <t>40V/2A</t>
   </si>
   <si>
@@ -348,12 +282,6 @@
     <t>SML-D12D1WT86</t>
   </si>
   <si>
-    <t xml:space="preserve">    D14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    D15</t>
-  </si>
-  <si>
     <t>ABLIC</t>
   </si>
   <si>
@@ -366,12 +294,6 @@
     <t>MCP73844T-840I/MS</t>
   </si>
   <si>
-    <t xml:space="preserve">    J4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    J6</t>
-  </si>
-  <si>
     <t>PJ-090BH</t>
   </si>
   <si>
@@ -387,15 +309,6 @@
     <t>TSM500P02CX RFG</t>
   </si>
   <si>
-    <t xml:space="preserve">    R2</t>
-  </si>
-  <si>
-    <t>&gt;  R3, R4</t>
-  </si>
-  <si>
-    <t>&gt;  R7-R9</t>
-  </si>
-  <si>
     <t xml:space="preserve">CR0603-FX-6200ELF </t>
   </si>
   <si>
@@ -417,21 +330,6 @@
     <t xml:space="preserve">ERJ-6RQFR22V </t>
   </si>
   <si>
-    <t xml:space="preserve">    R23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    R24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    R25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    R28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    R29</t>
-  </si>
-  <si>
     <t>User_Button</t>
   </si>
   <si>
@@ -444,42 +342,18 @@
     <t>B3U-1000P</t>
   </si>
   <si>
-    <t xml:space="preserve">    SW6</t>
-  </si>
-  <si>
     <t>ESP32-S3-WROOM-1</t>
   </si>
   <si>
     <t>espressif</t>
   </si>
   <si>
-    <t>&gt;  SW2-SW5, SW7</t>
-  </si>
-  <si>
     <t>EG1257</t>
   </si>
   <si>
     <t>PMOS_GSD-TSM260P02CX RFG</t>
   </si>
   <si>
-    <t>v3.0</t>
-  </si>
-  <si>
-    <t>&gt;  C1, C12, C15</t>
-  </si>
-  <si>
-    <t>&gt;  C2, C7, C9, C11, C13, C14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    C3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    C4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    C5</t>
-  </si>
-  <si>
     <t>2.2u</t>
   </si>
   <si>
@@ -495,54 +369,27 @@
     <t xml:space="preserve">GRM21BR61E226ME44K </t>
   </si>
   <si>
-    <t xml:space="preserve">    C16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    D5</t>
-  </si>
-  <si>
-    <t>&gt;  D6, D9, D10</t>
-  </si>
-  <si>
     <t>20V 1A</t>
   </si>
   <si>
     <t>SD0805S020S1R0</t>
   </si>
   <si>
-    <t>&gt;  D7, D8</t>
-  </si>
-  <si>
     <t>SD03C-7</t>
   </si>
   <si>
-    <t xml:space="preserve">    D11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    D12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    D13</t>
-  </si>
-  <si>
     <t>USB_C_Receptacle_USB2.0_16P</t>
   </si>
   <si>
     <t>2171820001</t>
   </si>
   <si>
-    <t xml:space="preserve">    J2</t>
-  </si>
-  <si>
     <t>Conn_02x11_Odd_Even</t>
   </si>
   <si>
     <t>TSM-111-01-T-DV</t>
   </si>
   <si>
-    <t xml:space="preserve">    J3</t>
-  </si>
-  <si>
     <t>Conn_02x05_Odd_Even</t>
   </si>
   <si>
@@ -567,70 +414,22 @@
     <t xml:space="preserve">SRP7050WA-220M </t>
   </si>
   <si>
-    <t xml:space="preserve">    L2</t>
-  </si>
-  <si>
     <t>TDK</t>
   </si>
   <si>
     <t>BCL322515RT-150M-D</t>
   </si>
   <si>
-    <t xml:space="preserve">    Q2</t>
-  </si>
-  <si>
-    <t>&gt;  Q3, Q4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Q5</t>
-  </si>
-  <si>
-    <t>&gt;  R1, R5, R6, R10, R11, R16, R17</t>
-  </si>
-  <si>
-    <t>&gt;  R12, R13</t>
-  </si>
-  <si>
     <t>4.7k</t>
   </si>
   <si>
     <t xml:space="preserve">RT0603FRE134K7L </t>
   </si>
   <si>
-    <t>&gt;  R14, R15, R22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    R18</t>
-  </si>
-  <si>
-    <t>51k</t>
-  </si>
-  <si>
-    <t>RT0603BRD0751KL</t>
-  </si>
-  <si>
-    <t>22.1k</t>
-  </si>
-  <si>
-    <t>RT0603BRD0722K1L</t>
-  </si>
-  <si>
-    <t>&gt;  R20, R21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    R26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    R27</t>
-  </si>
-  <si>
     <t>TPS560430X3FDBVR</t>
   </si>
   <si>
     <t>Texas Instruments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    U5</t>
   </si>
   <si>
     <t>SSQ-111-21-F-D</t>
@@ -705,6 +504,189 @@
   </si>
   <si>
     <t xml:space="preserve">06035C152KAT2A </t>
+  </si>
+  <si>
+    <t>BT1, BT2</t>
+  </si>
+  <si>
+    <t>C1, C12, C15</t>
+  </si>
+  <si>
+    <t>C2, C7, C9, C11, C13, C14</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>C4</t>
+  </si>
+  <si>
+    <t>C5</t>
+  </si>
+  <si>
+    <t>C6</t>
+  </si>
+  <si>
+    <t>C8</t>
+  </si>
+  <si>
+    <t>C10</t>
+  </si>
+  <si>
+    <t>C16</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>D2</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>D4</t>
+  </si>
+  <si>
+    <t>D5</t>
+  </si>
+  <si>
+    <t>D6, D9, D10</t>
+  </si>
+  <si>
+    <t>D7, D8</t>
+  </si>
+  <si>
+    <t>D11</t>
+  </si>
+  <si>
+    <t>D12</t>
+  </si>
+  <si>
+    <t>Diotec Semiconductor</t>
+  </si>
+  <si>
+    <t>SD103BW</t>
+  </si>
+  <si>
+    <t>D13</t>
+  </si>
+  <si>
+    <t>D14</t>
+  </si>
+  <si>
+    <t>D15</t>
+  </si>
+  <si>
+    <t>F1</t>
+  </si>
+  <si>
+    <t>J1</t>
+  </si>
+  <si>
+    <t>J2</t>
+  </si>
+  <si>
+    <t>J3</t>
+  </si>
+  <si>
+    <t>J4</t>
+  </si>
+  <si>
+    <t>J5</t>
+  </si>
+  <si>
+    <t>J6</t>
+  </si>
+  <si>
+    <t>J7</t>
+  </si>
+  <si>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>L2</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>Q3, Q4</t>
+  </si>
+  <si>
+    <t>Q5</t>
+  </si>
+  <si>
+    <t>R1, R5, R6, R10, R11, R16, R17</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>R3, R4</t>
+  </si>
+  <si>
+    <t>R7-R9</t>
+  </si>
+  <si>
+    <t>R12, R13</t>
+  </si>
+  <si>
+    <t>R14, R15, R18, R22</t>
+  </si>
+  <si>
+    <t>R20, R21</t>
+  </si>
+  <si>
+    <t>R23</t>
+  </si>
+  <si>
+    <t>R24</t>
+  </si>
+  <si>
+    <t>R25</t>
+  </si>
+  <si>
+    <t>R26</t>
+  </si>
+  <si>
+    <t>R27</t>
+  </si>
+  <si>
+    <t>R28</t>
+  </si>
+  <si>
+    <t>R29</t>
+  </si>
+  <si>
+    <t>SW1, SW2, SW4-SW7, SW9</t>
+  </si>
+  <si>
+    <t>SW3</t>
+  </si>
+  <si>
+    <t>SW8</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>U3</t>
+  </si>
+  <si>
+    <t>U4</t>
+  </si>
+  <si>
+    <t>U5</t>
+  </si>
+  <si>
+    <t>v3.1</t>
   </si>
 </sst>
 </file>
@@ -847,8 +829,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A4:E73" totalsRowShown="0" dataDxfId="5">
-  <autoFilter ref="A4:E73" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A4:E71" totalsRowShown="0" dataDxfId="5">
+  <autoFilter ref="A4:E71" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Reference" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Value" dataDxfId="3"/>
@@ -1123,7 +1105,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:H73"/>
+  <dimension ref="A2:H71"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="51" bestFit="1" customWidth="1"/>
@@ -1143,10 +1125,10 @@
         <v>0</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>145</v>
+        <v>211</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.35">
@@ -1154,30 +1136,30 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="C4" t="s">
-        <v>69</v>
+        <v>52</v>
       </c>
       <c r="D4" t="s">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>66</v>
+        <v>151</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="D5" s="3">
         <v>1043</v>
@@ -1188,16 +1170,16 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>95</v>
-      </c>
       <c r="D6" s="4" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="E6" s="5">
         <v>3</v>
@@ -1206,7 +1188,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>11</v>
@@ -1224,16 +1206,16 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="E8" s="5">
         <v>1</v>
@@ -1242,16 +1224,16 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>216</v>
-      </c>
       <c r="D9" s="4" t="s">
-        <v>217</v>
+        <v>150</v>
       </c>
       <c r="E9" s="5">
         <v>1</v>
@@ -1260,16 +1242,16 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>151</v>
+        <v>109</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>152</v>
+        <v>110</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>153</v>
+        <v>111</v>
       </c>
       <c r="E10" s="5">
         <v>1</v>
@@ -1278,10 +1260,10 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>97</v>
+        <v>157</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>5</v>
@@ -1296,16 +1278,16 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>98</v>
+        <v>158</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>214</v>
+        <v>147</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>154</v>
+        <v>112</v>
       </c>
       <c r="E12" s="5">
         <v>1</v>
@@ -1314,16 +1296,16 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>99</v>
+        <v>159</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>152</v>
+        <v>110</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>155</v>
+        <v>113</v>
       </c>
       <c r="E13" s="5">
         <v>1</v>
@@ -1332,7 +1314,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>14</v>
@@ -1350,16 +1332,16 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>16</v>
+        <v>161</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E15" s="5">
         <v>1</v>
@@ -1368,16 +1350,16 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>17</v>
+        <v>162</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="E16" s="5">
         <v>1</v>
@@ -1386,16 +1368,16 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>20</v>
+        <v>163</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E17" s="5">
         <v>1</v>
@@ -1404,16 +1386,16 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>101</v>
+        <v>164</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E18" s="5">
         <v>1</v>
@@ -1422,16 +1404,16 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E19" s="5">
         <v>1</v>
@@ -1440,16 +1422,16 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>159</v>
+        <v>114</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>214</v>
+        <v>147</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>160</v>
+        <v>115</v>
       </c>
       <c r="E20" s="5">
         <v>3</v>
@@ -1458,16 +1440,16 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>162</v>
+        <v>116</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>162</v>
+        <v>116</v>
       </c>
       <c r="E21" s="5">
         <v>2</v>
@@ -1476,13 +1458,13 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>214</v>
+        <v>147</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>6</v>
@@ -1494,16 +1476,16 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>18</v>
+        <v>170</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>19</v>
+        <v>171</v>
       </c>
       <c r="E23" s="5">
         <v>1</v>
@@ -1512,16 +1494,16 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>103</v>
+        <v>81</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>104</v>
+        <v>82</v>
       </c>
       <c r="E24" s="5">
         <v>1</v>
@@ -1530,16 +1512,16 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>107</v>
+        <v>173</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>105</v>
+        <v>83</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>106</v>
+        <v>84</v>
       </c>
       <c r="E25" s="5">
         <v>1</v>
@@ -1548,16 +1530,16 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>108</v>
+        <v>174</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E26" s="5">
         <v>1</v>
@@ -1566,10 +1548,10 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>32</v>
+        <v>175</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>1</v>
@@ -1584,16 +1566,16 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>34</v>
+        <v>176</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>166</v>
+        <v>117</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>167</v>
+        <v>118</v>
       </c>
       <c r="E28" s="5">
         <v>1</v>
@@ -1602,16 +1584,16 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>169</v>
+        <v>119</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>170</v>
+        <v>120</v>
       </c>
       <c r="E29" s="5">
         <v>1</v>
@@ -1620,16 +1602,16 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>172</v>
+        <v>121</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>173</v>
+        <v>122</v>
       </c>
       <c r="E30" s="5">
         <v>1</v>
@@ -1638,16 +1620,16 @@
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>113</v>
+        <v>179</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>174</v>
+        <v>123</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>175</v>
+        <v>124</v>
       </c>
       <c r="E31" s="5">
         <v>1</v>
@@ -1656,16 +1638,16 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>37</v>
+        <v>180</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>176</v>
+        <v>125</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>177</v>
+        <v>126</v>
       </c>
       <c r="E32" s="5">
         <v>1</v>
@@ -1674,16 +1656,16 @@
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>114</v>
+        <v>181</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>176</v>
+        <v>125</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>178</v>
+        <v>127</v>
       </c>
       <c r="E33" s="5">
         <v>1</v>
@@ -1692,16 +1674,16 @@
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>38</v>
+        <v>182</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>115</v>
+        <v>89</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>116</v>
+        <v>90</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>115</v>
+        <v>89</v>
       </c>
       <c r="E34" s="5">
         <v>1</v>
@@ -1710,16 +1692,16 @@
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>39</v>
+        <v>183</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>179</v>
+        <v>128</v>
       </c>
       <c r="E35" s="5">
         <v>1</v>
@@ -1728,16 +1710,16 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>181</v>
+        <v>129</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>182</v>
+        <v>130</v>
       </c>
       <c r="E36" s="5">
         <v>1</v>
@@ -1745,16 +1727,16 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>40</v>
+        <v>185</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="E37" s="5">
         <v>1</v>
@@ -1763,16 +1745,16 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>144</v>
+        <v>108</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="E38" s="5">
         <v>1</v>
@@ -1781,16 +1763,16 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E39" s="5">
         <v>2</v>
@@ -1798,16 +1780,16 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>117</v>
+        <v>91</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>118</v>
+        <v>92</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>119</v>
+        <v>93</v>
       </c>
       <c r="E40" s="5">
         <v>1</v>
@@ -1815,16 +1797,16 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="E41" s="5">
         <v>7</v>
@@ -1832,7 +1814,7 @@
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>120</v>
+        <v>190</v>
       </c>
       <c r="B42" s="3">
         <v>300</v>
@@ -1841,7 +1823,7 @@
         <v>1</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="E42" s="5">
         <v>1</v>
@@ -1849,7 +1831,7 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>121</v>
+        <v>191</v>
       </c>
       <c r="B43" s="3">
         <v>100</v>
@@ -1858,7 +1840,7 @@
         <v>12</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="E43" s="5">
         <v>2</v>
@@ -1866,16 +1848,16 @@
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>122</v>
+        <v>192</v>
       </c>
       <c r="B44" s="3">
         <v>620</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>123</v>
+        <v>94</v>
       </c>
       <c r="E44" s="5">
         <v>3</v>
@@ -1883,16 +1865,16 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>188</v>
+        <v>131</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>189</v>
+        <v>132</v>
       </c>
       <c r="E45" s="5">
         <v>2</v>
@@ -1900,7 +1882,7 @@
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B46" s="3">
         <v>0</v>
@@ -1909,41 +1891,41 @@
         <v>12</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="E46" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>192</v>
+        <v>195</v>
+      </c>
+      <c r="B47" s="3">
+        <v>470</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>193</v>
+        <v>40</v>
       </c>
       <c r="E47" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>79</v>
+        <v>196</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>194</v>
+        <v>95</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>12</v>
+        <v>96</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>195</v>
+        <v>97</v>
       </c>
       <c r="E48" s="5">
         <v>1</v>
@@ -1951,33 +1933,33 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="B49" s="3">
-        <v>470</v>
+        <v>197</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>98</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>46</v>
+        <v>99</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>51</v>
+        <v>100</v>
       </c>
       <c r="E49" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>124</v>
+        <v>198</v>
+      </c>
+      <c r="B50" s="3">
+        <v>0</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>125</v>
+        <v>12</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>126</v>
+        <v>54</v>
       </c>
       <c r="E50" s="5">
         <v>1</v>
@@ -1985,16 +1967,16 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>131</v>
+        <v>199</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>127</v>
+        <v>41</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>128</v>
+        <v>12</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>129</v>
+        <v>42</v>
       </c>
       <c r="E51" s="5">
         <v>1</v>
@@ -2002,16 +1984,16 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="B52" s="3">
-        <v>0</v>
+        <v>200</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>69</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>71</v>
+        <v>148</v>
       </c>
       <c r="E52" s="5">
         <v>1</v>
@@ -2019,16 +2001,16 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="C53" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="E53" s="5">
         <v>1</v>
@@ -2036,16 +2018,16 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>87</v>
+        <v>38</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>215</v>
+        <v>39</v>
       </c>
       <c r="E54" s="5">
         <v>1</v>
@@ -2053,33 +2035,33 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>133</v>
+        <v>203</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>54</v>
+        <v>102</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>12</v>
+        <v>103</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>55</v>
+        <v>104</v>
       </c>
       <c r="E55" s="5">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>134</v>
+        <v>204</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>49</v>
+        <v>101</v>
       </c>
       <c r="C56" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D56" s="3" t="s">
         <v>46</v>
-      </c>
-      <c r="D56" s="3" t="s">
-        <v>50</v>
       </c>
       <c r="E56" s="5">
         <v>1</v>
@@ -2087,16 +2069,16 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>57</v>
+        <v>205</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>135</v>
+        <v>107</v>
       </c>
       <c r="C57" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>58</v>
+        <v>107</v>
       </c>
       <c r="E57" s="5">
         <v>1</v>
@@ -2104,33 +2086,33 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>142</v>
+        <v>206</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>136</v>
+        <v>105</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>137</v>
+        <v>106</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>138</v>
+        <v>105</v>
       </c>
       <c r="E58" s="5">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>139</v>
+        <v>207</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>143</v>
+        <v>47</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>143</v>
+        <v>47</v>
       </c>
       <c r="E59" s="5">
         <v>1</v>
@@ -2138,16 +2120,16 @@
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>59</v>
+        <v>208</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="E60" s="5">
         <v>1</v>
@@ -2155,16 +2137,16 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>62</v>
+        <v>209</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="E61" s="5">
         <v>1</v>
@@ -2172,90 +2154,90 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>63</v>
+        <v>210</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>199</v>
+        <v>86</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>200</v>
+        <v>87</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>199</v>
+        <v>88</v>
       </c>
       <c r="E62" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B63" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C63" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="D63" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="E63" s="5">
-        <v>1</v>
-      </c>
+      <c r="A63" s="3"/>
+      <c r="B63" s="3"/>
+      <c r="C63" s="3"/>
+      <c r="D63" s="3"/>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>201</v>
+        <v>58</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>110</v>
+        <v>56</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>112</v>
+        <v>57</v>
+      </c>
+      <c r="D64" s="3">
+        <v>100833</v>
       </c>
       <c r="E64" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" s="3"/>
-      <c r="B65" s="3"/>
-      <c r="C65" s="3"/>
-      <c r="D65" s="3"/>
+      <c r="A65" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B65" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D65" t="s">
+        <v>135</v>
+      </c>
+      <c r="E65" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>73</v>
+        <v>138</v>
+      </c>
+      <c r="B66" s="9" t="s">
+        <v>144</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="D66" s="3">
-        <v>100833</v>
+        <v>29</v>
+      </c>
+      <c r="D66" t="s">
+        <v>136</v>
       </c>
       <c r="E66" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="B67" s="9" t="s">
-        <v>210</v>
+        <v>139</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>145</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D67" t="s">
-        <v>202</v>
+        <v>140</v>
       </c>
       <c r="E67" s="5">
         <v>1</v>
@@ -2263,72 +2245,38 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="B68" s="9" t="s">
-        <v>211</v>
+        <v>142</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>146</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D68" t="s">
-        <v>203</v>
+        <v>141</v>
       </c>
       <c r="E68" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="C69" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D69" t="s">
-        <v>207</v>
-      </c>
-      <c r="E69" s="5">
-        <v>1</v>
-      </c>
+      <c r="A69" s="3"/>
+      <c r="B69" s="3"/>
+      <c r="C69" s="3"/>
+      <c r="D69" s="8"/>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D70" t="s">
-        <v>208</v>
-      </c>
-      <c r="E70" s="5">
-        <v>1</v>
-      </c>
+      <c r="A70" s="3"/>
+      <c r="B70" s="3"/>
+      <c r="C70" s="3"/>
+      <c r="D70" s="3"/>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
       <c r="C71" s="3"/>
-      <c r="D71" s="8"/>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="3"/>
-      <c r="B72" s="3"/>
-      <c r="C72" s="3"/>
-      <c r="D72" s="3"/>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" s="3"/>
-      <c r="B73" s="3"/>
-      <c r="C73" s="3"/>
-      <c r="D73" s="3"/>
+      <c r="D71" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>